<commit_message>
Update LencoAbroad With Chat Rooms
</commit_message>
<xml_diff>
--- a/backend/chatdata/CR-1001.xlsx
+++ b/backend/chatdata/CR-1001.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -519,9 +519,69 @@
         <v>5/10/2026, 10:32:15 AM</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Chunilal Bhut</v>
+      </c>
+      <c r="B7" t="str">
+        <v>csbhut11</v>
+      </c>
+      <c r="C7" t="str">
+        <v>11111</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v>8/16/2026, 9:33:52 AM</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Chunilal Bhut</v>
+      </c>
+      <c r="B8" t="str">
+        <v>csbhut11</v>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v>CR-1001_1786887243308.JPG</v>
+      </c>
+      <c r="E8" t="str">
+        <v>image/jpeg</v>
+      </c>
+      <c r="F8" t="str">
+        <v>8/16/2026, 9:34:03 AM</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Chunilal Bhut</v>
+      </c>
+      <c r="B9" t="str">
+        <v>csbhut11</v>
+      </c>
+      <c r="C9" t="str">
+        <v>I need to join this website વેબસાઈટ જોઈન કરવી છે इस वेबसाइट ज्वाइन करना चाहता हूं</v>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v>8/16/2026, 9:34:36 AM</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>